<commit_message>
chore(i18n): refresh Latvian from complete translations-review.xlsx
Regenerated messages/lv.json via scripts/apply-lv-from-xlsx.mjs; workbook column E is now fully filled for translatable copy.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/translations-review.xlsx
+++ b/translations-review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sascha/Nordora Vital SIA/Website/web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB609D1-7BF5-4046-8348-72107BFFDE14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E743748-17E1-A54B-B703-7EA6B19C8665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43780" yWindow="-8560" windowWidth="37660" windowHeight="26980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46220" yWindow="-8560" windowWidth="35220" windowHeight="26980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Translations" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3663" uniqueCount="2642">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3663" uniqueCount="2736">
   <si>
     <t>Location / context</t>
   </si>
@@ -7609,9 +7609,6 @@
     <t>Piedāvājiet to pašu labklājības iespēju arī personālam — īsus brīžus starp sarakstiem — lai atbalstītu komandas morāli, nesajaucot to ar arodveselības pakalpojumiem.</t>
   </si>
   <si>
-    <t>Pārejas posmos izmantojama apsējs locītavām vai ekstremitātēm.</t>
-  </si>
-  <si>
     <t>Attēls: {product} — sanza labsajūtas modulis profesionālai lietošanai telpās.</t>
   </si>
   <si>
@@ -7988,19 +7985,310 @@
   </si>
   <si>
     <t>Piedāvājiet ikmēneša abonementu, lai piekļūtu labsajūtas atpūtas telpai, kas aprīkota ar &lt;strong&gt;sanza&lt;/strong&gt; — īsām sesijām, ko klienti var izmantot pirms vai starp vizītēm, vai atveseļošanās dienās.</t>
+  </si>
+  <si>
+    <t>Lokālie aplikatori īsiem, mērķtiecīgiem komforta brīžiem — žoklim/kaklam/pleciem, ekstremitātēm vai zonām, kas saglabā sasprindzinājumu. Ideāli piemēroti kā “ierašanās rīks” vai mierīgam noslēgumam pēc vizītes — stingri ievērojot vispārējo labsajūtas pozīciju.</t>
+  </si>
+  <si>
+    <t>Īsi, precīzi, viegli integrējami.</t>
+  </si>
+  <si>
+    <t>&lt;strong&gt;sanza&lt;/strong&gt; iestatīšana, ko jūsu komanda var izmantot — katru dienu</t>
+  </si>
+  <si>
+    <t>&lt;strong&gt;sanza&lt;/strong&gt; ir izstrādāta reālām klīnikām un praksēm: vienkārša aparatūra, skaidras programmas un konsekventa secība, ko jūsu komanda var nodrošināt bez minējumiem. Jūs saņemat vienu sistēmu, kas atbalsta komfortu un mierīgāku vizīti, kamēr jūsu klīniskais darbs paliek tieši tur, kur tam jābūt: centrā.</t>
+  </si>
+  <si>
+    <t>Viens vadības centrs laika noteikšanai, programmām un secībai.</t>
+  </si>
+  <si>
+    <t>Iestatiet plūsmu vienreiz un pēc tam droši palaidiet to — pat noslogotās dienās un vairākās telpās.</t>
+  </si>
+  <si>
+    <t>Visa ķermeņa + lokālas opcijas dažādiem vizītes brīžiem.</t>
+  </si>
+  <si>
+    <t>Izmantojiet to ierašanās brīdim, īsai pauzei vizītes vidū vai mierīgam noslēgumam — nepagarinot vizītes ilgumu.</t>
+  </si>
+  <si>
+    <t>15 numurētas programmas, kas nodrošina konsekventu izpildi.</t>
+  </si>
+  <si>
+    <t>Personālam viegli apgūstams, viegli atkārtojams — lai pieredze šķistu “kā jūsu prakse”, nevis kā ierīce.</t>
+  </si>
+  <si>
+    <t>Papildu aplikatori īsiem, mērķtiecīgiem komforta brīžiem.</t>
+  </si>
+  <si>
+    <t>Ātri pieskāriena punkti, kur cilvēki saglabā spriedzi — izstrādāti, lai netraucēti integrētos jūsu ikdienas rutīnā.</t>
+  </si>
+  <si>
+    <t>Sanza sistēmas pārskats — modulārs profesionāls labsajūtas aprīkojums.</t>
+  </si>
+  <si>
+    <t>Ģenerators</t>
+  </si>
+  <si>
+    <t>Paklājiņš</t>
+  </si>
+  <si>
+    <t>Paliktnis</t>
+  </si>
+  <si>
+    <t>Pildspalva</t>
+  </si>
+  <si>
+    <t>Kas mainās klientiem — un jūsu komandai</t>
+  </si>
+  <si>
+    <t>Vienkārša valoda. Tikai labsajūtas efekti telpās: komforts, miers, vienmērīgāka plūsma — bez medicīniskiem solījumiem.</t>
+  </si>
+  <si>
+    <t>Piedāvātie pakalpojumi</t>
+  </si>
+  <si>
+    <t>Mierīgāka ierašanās</t>
+  </si>
+  <si>
+    <t>Biofrekvences programmas — vadītā atiestatīšana</t>
+  </si>
+  <si>
+    <t>Biofrekvences programmas tiek piegādātas, izmantojot rokas elektrodus. Klienti tos tur īsas programmas laikā — vienkārša, sēdus un viegli izpildāma. Uztveriet to kā vadītu labsajūtas rutīnu, kas padara pieredzi apzinātu un strukturētu.</t>
+  </si>
+  <si>
+    <t>Zinātniskais pamatojums</t>
+  </si>
+  <si>
+    <t>Tie ir zemas intensitātes bioelektriskās frekvences modeļi, kas tiek piegādāti, izmantojot kontakta elektrodus. Biofizikas literatūrā pielietotie elektriskie lauki tiek apspriesti saistībā ar šūnu membrānas potenciāliem un signalizāciju. Jūsu vidē vērtība ir praktiska: atkārtojama rutīna, kas atbalsta mierīgu koncentrēšanos un atiestatīšanas sajūtu, neprasot personālam improvizēt.</t>
+  </si>
+  <si>
+    <t>03 — AUKSTAIS LĀZERS</t>
+  </si>
+  <si>
+    <t>Aukstais lāzers — precīzs komforta pieskāriena punkts</t>
+  </si>
+  <si>
+    <t>Aukstais lāzers ir fotobiomodulācija: mērķtiecīga gaisma, kas lokāli tiek pielietota īsu laiku kā precīzs papildinājums. To bieži izmanto vietās, kur klienti saglabā sasprindzinājumu — žoklī, kaklā, plecos, ekstremitātēs — vai kā tīru noslēguma rituālu.</t>
+  </si>
+  <si>
+    <t>Fotobiomodulācija tiek plaši apspriesta saistībā ar mitohondriju aktivitāti un lokālo audu signalizāciju. Praktiski tas ir neinvazīvs veids, kā pievienot fokusētu lokālu mirkli, kas atbalsta komfortu un augstākās kvalitātes aprūpes sajūtu.</t>
+  </si>
+  <si>
+    <t>Jūs saglabājat savu metodi centrā. &lt;strong&gt;sanza&lt;/strong&gt; atbalsta apkārtējo stāvokli — ierašanos, tempu un noslēgumu —, lai vizīte šķistu mierīgāka, vienmērīgāka un neaizmirstamāka.</t>
+  </si>
+  <si>
+    <t>Lielākā daļa pacientu &lt;strong&gt;sanza&lt;/strong&gt; raksturo kā ievērojamu stāvokļa maiņu. Viņi ierodas enerģiski — saspringti, steidzīgi, pārlieku stimulēti — un dažu minūšu laikā jūt, kā viņu elpošana palēninās, pleci nolaižas un ķermenis nomierinās.</t>
+  </si>
+  <si>
+    <t>Ko viņi parasti pamana:</t>
+  </si>
+  <si>
+    <t>Mazāk stresa/iekšējā trokšņa — mierīgāka galvas telpa, mazāk saspringta</t>
+  </si>
+  <si>
+    <t>Vidējāka enerģija — iezemēta, līdzsvarota, nevis sedatīva</t>
+  </si>
+  <si>
+    <t>Lokāla atbrīvošanās — mērķtiecīga relaksācija vietās, kur atrodas sasprindzinājums (žoklis, kakls, pleci, ekstremitātes)</t>
+  </si>
+  <si>
+    <t>Mīkstāka piezemēšanās — viņi pēc vizītes aiziet mierīgāki, skaidrāki un ērtāk</t>
+  </si>
+  <si>
+    <t>Labsajūtas papildinājums jūsu praksei.</t>
+  </si>
+  <si>
+    <t>Tipiska &lt;strong&gt;sanza&lt;/strong&gt; iekārta ietver:</t>
+  </si>
+  <si>
+    <t>Ģenerators — divi augstas veiktspējas magnētiskie ģeneratori vienā ierīcē (divas izejas)</t>
+  </si>
+  <si>
+    <t>Jūs izmantojat &lt;strong&gt;sanza&lt;/strong&gt; iekšēji, lai atbalstītu savu komandu ar īsiem labsajūtas brīžiem visas dienas garumā.</t>
+  </si>
+  <si>
+    <t>Jūs varat to veidot kā daļu no savas iekšējās aprūpes kultūras — praktisku veidu, kā atbalstīt klātbūtni, stabilitāti un atmosfēras kvalitāti, ko jūsu klienti izjūt, ienākot.</t>
+  </si>
+  <si>
+    <t>Apskatiet, kā &lt;strong&gt;sanza&lt;/strong&gt; varētu izskatīties jūsu uzņēmumā.</t>
+  </si>
+  <si>
+    <t>Katra prakse ir atšķirīga. Tāpēc &lt;strong&gt;sanza&lt;/strong&gt; nav veidota ap vienu stingru modeli, bet gan ap pakalpojumu formātiem, kurus varat pielāgot klientu plūsmai, cenām un pozicionēšanai. Izmantojiet kalkulatoru, lai izpētītu, ko reālistiska &lt;strong&gt;sanza&lt;/strong&gt; integrācija varētu nozīmēt jūsu ikmēneša ieņēmumiem un atmaksāšanās periodam.</t>
+  </si>
+  <si>
+    <t>Klienti dienā (atbilstoši papildinājumam)</t>
+  </si>
+  <si>
+    <t>Darba dienas mēnesī</t>
+  </si>
+  <si>
+    <t>Pievienotās likmes (%)</t>
+  </si>
+  <si>
+    <t>Vidējā papildinājuma cena ({valūta})</t>
+  </si>
+  <si>
+    <t>Maksājošie atpūtas telpas biedri (mēnesī)</t>
+  </si>
+  <si>
+    <t>Dalības cena par biedru ({valūta}/mēnesī)</t>
+  </si>
+  <si>
+    <t>Pieņemtās aprīkojuma investīcijas ({valūta})</t>
+  </si>
+  <si>
+    <t>Fizioterapeitiem</t>
+  </si>
+  <si>
+    <t>Fizioterapeitiem, kas vēlas labsajūtas slāni ap nodarbībām — viegli vadīt, viegli izskaidrot, ērti novietot.</t>
+  </si>
+  <si>
+    <t>Ikona, kas norāda uz fizioterapiju un uz kustībām orientētu praksi līdzās labsajūtas tehnoloģijām.</t>
+  </si>
+  <si>
+    <t>Mēs skaidri norādām, ka **sanza** nav daļa no rehabilitācijas protokola — tā ir sagaidīšana un nomierināšanās.</t>
+  </si>
+  <si>
+    <t>Prakses īpašnieks, pagaidu darbinieks</t>
+  </si>
+  <si>
+    <t>Pacienti min, ka jūtas “pamanīti” — mūsu PROM nemainījās, bet gan apmierinātība gan.</t>
+  </si>
+  <si>
+    <t>Vadošais fizioterapeits, pagaidu darbinieks</t>
+  </si>
+  <si>
+    <t>Personāls lūdza tādu pašu mieru starp pacientiem pēc kārtas.</t>
+  </si>
+  <si>
+    <t>Klīnikas vadītājs, pagaidu darbinieks</t>
+  </si>
+  <si>
+    <t>Skatiet **sanza** līdzās savam klīniskajam darbam</t>
+  </si>
+  <si>
+    <t>Rezervējiet demonstrāciju vai pieprasiet pilotprojektu — mēs palīdzēsim jums skaidri formulēt rituālus pacientiem un regulatoriem.</t>
+  </si>
+  <si>
+    <t>Pieprasiet pilotprojektu</t>
+  </si>
+  <si>
+    <t>Dalieties ar savu kontekstu zemāk — mēs palīdzēsim jums plānot atdalīšanos no klīniskajām plūsmām.</t>
+  </si>
+  <si>
+    <t>Fizioterapeiti | Nordora Vital</t>
+  </si>
+  <si>
+    <t>Uzlabojiet prakses pieredzi ar sanza — nomierināšanās pirms sesijas un dekompresija pēc sesijas, kas neaizstāj rehabilitācijas protokolus vai klīniskos vingrinājumus.</t>
+  </si>
+  <si>
+    <t>Skatiet, kā moduļi savienojas mūsu sistēmas pārskatā — šeit nav publiskas aparatūras cenas.</t>
+  </si>
+  <si>
+    <t>Kompakts spilventiņš lokāliem komforta brīžiem.</t>
+  </si>
+  <si>
+    <t>Aptinums locītavām vai ekstremitātēm pārejas laikā.</t>
+  </si>
+  <si>
+    <t>Izveidojiet atsevišķu labsajūtas atpūtas telpu vai kluso zonu ierašanās un dekompresijas rituāliem — fiziski un operacionāli atdalītu no izmeklēšanas un ārstēšanas plūsmām.</t>
+  </si>
+  <si>
+    <t>Izmantojiet ROI un komplekso domāšanu: apvienojiet piekļuvi atpūtas telpai, sesiju paketes un dalību, lai atkārtotie ieņēmumi atbalstītu ieguldījumus — formātus skatiet arī mūsu Piedāvājumu lapā.</t>
+  </si>
+  <si>
+    <t>Piedāvājiet personālam piekļuvi labsajūtai vienā un tajā pašā atpūtas telpas modelī — noturēšanas un kultūras priekšrocības, kas netraucē klīniskajiem pienākumiem vai sterilām zonām.</t>
+  </si>
+  <si>
+    <t>Ko saka vadītāji</t>
+  </si>
+  <si>
+    <t>Mēs palielinājām ieņēmumus, nemainot nevienu klīnisko SOP — tieši to, ko valde vēlējās dzirdēt.</t>
+  </si>
+  <si>
+    <t>Biedru skaits pieauga, kad atpūtas telpai bija nosaukums un grafiks.</t>
+  </si>
+  <si>
+    <t>Klīnikas operāciju direktors, pagaidu darbinieks</t>
+  </si>
+  <si>
+    <t>Pacienti beidz to saukt par "tikai uzgaidāmo telpu" — tas ir bijis izmēģinājuma projekta vērts.</t>
+  </si>
+  <si>
+    <t>Operāciju direktors, pagaidu darbinieks</t>
+  </si>
+  <si>
+    <t>Plānojiet labsajūtas slāni ar Nordora Vital</t>
+  </si>
+  <si>
+    <t>Rezervējiet demonstrāciju vai pieprasiet izmēģinājuma projektu — mēs saskaņosim atpūtas telpas dizainu, pārvaldību un ekonomiku ar jūsu ietekmi.</t>
+  </si>
+  <si>
+    <t>Zemāk izklāstiet savus mērķus — mēs jūs savienosim ar ekonomiku, atpūtas telpas dizainu un ieviešanas iespējām. Klīniku un prakšu īpašnieki | Nordora Vital</t>
+  </si>
+  <si>
+    <t>Pievienojiet īpašu labsajūtas atpūtas telpu vai augstākās klases komforta slāni — ROI domāšanu, dalību un personāla labsajūtu —, nemainot klīniskos protokolus.</t>
+  </si>
+  <si>
+    <t>Pievienojiet īpašu labsajūtas atpūtas telpu vai augstākās klases komforta slāni — ROI domāšanu, dalību un darbinieku labsajūtu —, nemainot klīniskos protokolus.</t>
+  </si>
+  <si>
+    <t>Labsajūtas atpūtas telpas vai dalības piekļuves koncepcijas ilustrācija regulāriem labsajūtas apmeklējumiem.</t>
+  </si>
+  <si>
+    <t>ATKĀRTOTI IEŅĒMUMI</t>
+  </si>
+  <si>
+    <t>Dalībību līmeņi (piemēram, tikai atpūtas telpa vs. atpūtas telpa + ikmēneša papildu kredīti), lai atbilstu dažādiem klientu tēriņu līmeņiem.</t>
+  </si>
+  <si>
+    <t>Atkārtota dalība rada paredzamus ieņēmumus un stiprina lojalitāti, kad biedri piedzīvo vienmērīgu tempu un atmosfēru.</t>
+  </si>
+  <si>
+    <t>Dalība/atveseļošanās atpūtas telpa</t>
+  </si>
+  <si>
+    <t>INVESTĪCIJU ATDEVE</t>
+  </si>
+  <si>
+    <t>Pozicionējiet to kā darbinieku priekšrocību līdzās apmācībām un ergonomikai: izvēles, izvēles un saskaņota ar vispārējo labsajūtu, nevis arodslimību prasībām.</t>
+  </si>
+  <si>
+    <t>Izmantojiet sistēmu iekšēji savai komandai — īsas sesijas starp maiņām vai pārtraukumos —, lai atbalstītu koncentrēšanos, mierīgas pārejas un pozitīvu darba vietas kultūru.</t>
+  </si>
+  <si>
+    <t>Ilustrācija, kurā darbinieki izmanto īsus labsajūtas pārtraukumus starp maiņām profesionālā darba vietā.</t>
+  </si>
+  <si>
+    <t>KOMANDAS LABKLĀJĪBA</t>
+  </si>
+  <si>
+    <t>Izmaksas var piešķirt personāla vadības vai apmācību budžetiem; netiešā atdeve rodas no iesaistes, noturēšanas un ar klientu vērstas enerģijas konsekvences.</t>
+  </si>
+  <si>
+    <t>Darbinieku labsajūtas plāns</t>
+  </si>
+  <si>
+    <t>Izvēlieties savu nozari</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -8023,11 +8311,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9595,8 +9884,8 @@
       <c r="D72" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="E72" s="1" t="s">
-        <v>279</v>
+      <c r="E72" s="2" t="s">
+        <v>2641</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9612,8 +9901,8 @@
       <c r="D73" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="E73" s="1" t="s">
-        <v>283</v>
+      <c r="E73" s="2" t="s">
+        <v>2642</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9629,8 +9918,8 @@
       <c r="D74" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="E74" s="1" t="s">
-        <v>287</v>
+      <c r="E74" s="2" t="s">
+        <v>2643</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -9646,8 +9935,8 @@
       <c r="D75" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="E75" s="1" t="s">
-        <v>291</v>
+      <c r="E75" s="2" t="s">
+        <v>2644</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9663,8 +9952,8 @@
       <c r="D76" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="E76" s="1" t="s">
-        <v>295</v>
+      <c r="E76" s="2" t="s">
+        <v>2645</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -9680,8 +9969,8 @@
       <c r="D77" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="E77" s="1" t="s">
-        <v>299</v>
+      <c r="E77" s="2" t="s">
+        <v>2646</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9697,8 +9986,8 @@
       <c r="D78" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="E78" s="1" t="s">
-        <v>303</v>
+      <c r="E78" s="2" t="s">
+        <v>2647</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -9714,8 +10003,8 @@
       <c r="D79" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="E79" s="1" t="s">
-        <v>307</v>
+      <c r="E79" s="2" t="s">
+        <v>2648</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9731,8 +10020,8 @@
       <c r="D80" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E80" s="1" t="s">
-        <v>311</v>
+      <c r="E80" s="2" t="s">
+        <v>2649</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -9748,8 +10037,8 @@
       <c r="D81" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="E81" s="1" t="s">
-        <v>315</v>
+      <c r="E81" s="2" t="s">
+        <v>2650</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9765,8 +10054,8 @@
       <c r="D82" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="E82" s="1" t="s">
-        <v>319</v>
+      <c r="E82" s="2" t="s">
+        <v>2651</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -9782,8 +10071,8 @@
       <c r="D83" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E83" s="1" t="s">
-        <v>323</v>
+      <c r="E83" s="2" t="s">
+        <v>2652</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9799,8 +10088,8 @@
       <c r="D84" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="E84" s="1" t="s">
-        <v>327</v>
+      <c r="E84" s="2" t="s">
+        <v>2653</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9816,8 +10105,8 @@
       <c r="D85" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="E85" s="1" t="s">
-        <v>331</v>
+      <c r="E85" s="2" t="s">
+        <v>2654</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9833,8 +10122,8 @@
       <c r="D86" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="E86" s="1" t="s">
-        <v>333</v>
+      <c r="E86" s="2" t="s">
+        <v>2655</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9850,8 +10139,8 @@
       <c r="D87" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="E87" s="1" t="s">
-        <v>335</v>
+      <c r="E87" s="2" t="s">
+        <v>2656</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9867,8 +10156,8 @@
       <c r="D88" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="E88" s="1" t="s">
-        <v>337</v>
+      <c r="E88" s="2" t="s">
+        <v>2657</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9884,8 +10173,8 @@
       <c r="D89" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="E89" s="1" t="s">
-        <v>340</v>
+      <c r="E89" s="2" t="s">
+        <v>2658</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -9901,8 +10190,8 @@
       <c r="D90" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="E90" s="1" t="s">
-        <v>344</v>
+      <c r="E90" s="2" t="s">
+        <v>2659</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9918,8 +10207,8 @@
       <c r="D91" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="E91" s="1" t="s">
-        <v>348</v>
+      <c r="E91" s="2" t="s">
+        <v>2660</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -9935,8 +10224,8 @@
       <c r="D92" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="E92" s="1" t="s">
-        <v>351</v>
+      <c r="E92" s="2" t="s">
+        <v>2661</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11227,8 +11516,8 @@
       <c r="D168" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="E168" s="1" t="s">
-        <v>667</v>
+      <c r="E168" s="2" t="s">
+        <v>2662</v>
       </c>
     </row>
     <row r="169" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11244,8 +11533,8 @@
       <c r="D169" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="E169" s="1" t="s">
-        <v>645</v>
+      <c r="E169" s="2" t="s">
+        <v>647</v>
       </c>
     </row>
     <row r="170" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -11261,8 +11550,8 @@
       <c r="D170" s="1" t="s">
         <v>674</v>
       </c>
-      <c r="E170" s="1" t="s">
-        <v>673</v>
+      <c r="E170" s="2" t="s">
+        <v>2663</v>
       </c>
     </row>
     <row r="171" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11278,8 +11567,8 @@
       <c r="D171" s="1" t="s">
         <v>655</v>
       </c>
-      <c r="E171" s="1" t="s">
-        <v>654</v>
+      <c r="E171" s="2" t="s">
+        <v>2664</v>
       </c>
     </row>
     <row r="172" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -11295,8 +11584,8 @@
       <c r="D172" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="E172" s="1" t="s">
-        <v>679</v>
+      <c r="E172" s="2" t="s">
+        <v>2665</v>
       </c>
     </row>
     <row r="173" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11312,8 +11601,8 @@
       <c r="D173" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="E173" s="1" t="s">
-        <v>683</v>
+      <c r="E173" s="2" t="s">
+        <v>2666</v>
       </c>
     </row>
     <row r="174" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11329,8 +11618,8 @@
       <c r="D174" s="1" t="s">
         <v>688</v>
       </c>
-      <c r="E174" s="1" t="s">
-        <v>687</v>
+      <c r="E174" s="2" t="s">
+        <v>2667</v>
       </c>
     </row>
     <row r="175" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11346,8 +11635,8 @@
       <c r="D175" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="E175" s="1" t="s">
-        <v>645</v>
+      <c r="E175" s="2" t="s">
+        <v>647</v>
       </c>
     </row>
     <row r="176" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -11363,8 +11652,8 @@
       <c r="D176" s="1" t="s">
         <v>694</v>
       </c>
-      <c r="E176" s="1" t="s">
-        <v>693</v>
+      <c r="E176" s="2" t="s">
+        <v>2668</v>
       </c>
     </row>
     <row r="177" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11380,8 +11669,8 @@
       <c r="D177" s="1" t="s">
         <v>655</v>
       </c>
-      <c r="E177" s="1" t="s">
-        <v>654</v>
+      <c r="E177" s="2" t="s">
+        <v>2664</v>
       </c>
     </row>
     <row r="178" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -11397,8 +11686,8 @@
       <c r="D178" s="1" t="s">
         <v>700</v>
       </c>
-      <c r="E178" s="1" t="s">
-        <v>699</v>
+      <c r="E178" s="2" t="s">
+        <v>2669</v>
       </c>
     </row>
     <row r="179" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -11414,8 +11703,8 @@
       <c r="D179" s="1" t="s">
         <v>704</v>
       </c>
-      <c r="E179" s="1" t="s">
-        <v>703</v>
+      <c r="E179" s="2" t="s">
+        <v>2670</v>
       </c>
     </row>
     <row r="180" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -11431,8 +11720,8 @@
       <c r="D180" s="1" t="s">
         <v>708</v>
       </c>
-      <c r="E180" s="1" t="s">
-        <v>707</v>
+      <c r="E180" s="2" t="s">
+        <v>2671</v>
       </c>
     </row>
     <row r="181" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11448,8 +11737,8 @@
       <c r="D181" s="1" t="s">
         <v>712</v>
       </c>
-      <c r="E181" s="1" t="s">
-        <v>711</v>
+      <c r="E181" s="2" t="s">
+        <v>2672</v>
       </c>
     </row>
     <row r="182" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11465,8 +11754,8 @@
       <c r="D182" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="E182" s="1" t="s">
-        <v>715</v>
+      <c r="E182" s="2" t="s">
+        <v>2673</v>
       </c>
     </row>
     <row r="183" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11482,8 +11771,8 @@
       <c r="D183" s="1" t="s">
         <v>720</v>
       </c>
-      <c r="E183" s="1" t="s">
-        <v>719</v>
+      <c r="E183" s="2" t="s">
+        <v>2674</v>
       </c>
     </row>
     <row r="184" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11499,8 +11788,8 @@
       <c r="D184" s="1" t="s">
         <v>724</v>
       </c>
-      <c r="E184" s="1" t="s">
-        <v>723</v>
+      <c r="E184" s="2" t="s">
+        <v>2675</v>
       </c>
     </row>
     <row r="185" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11516,8 +11805,8 @@
       <c r="D185" s="1" t="s">
         <v>728</v>
       </c>
-      <c r="E185" s="1" t="s">
-        <v>727</v>
+      <c r="E185" s="2" t="s">
+        <v>2676</v>
       </c>
     </row>
     <row r="186" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11533,8 +11822,8 @@
       <c r="D186" s="1" t="s">
         <v>732</v>
       </c>
-      <c r="E186" s="1" t="s">
-        <v>731</v>
+      <c r="E186" s="2" t="s">
+        <v>2677</v>
       </c>
     </row>
     <row r="187" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -11550,8 +11839,8 @@
       <c r="D187" s="1" t="s">
         <v>736</v>
       </c>
-      <c r="E187" s="1" t="s">
-        <v>735</v>
+      <c r="E187" s="2" t="s">
+        <v>2678</v>
       </c>
     </row>
     <row r="188" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -11567,8 +11856,8 @@
       <c r="D188" s="1" t="s">
         <v>740</v>
       </c>
-      <c r="E188" s="1" t="s">
-        <v>739</v>
+      <c r="E188" s="2" t="s">
+        <v>2679</v>
       </c>
     </row>
     <row r="189" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12145,8 +12434,8 @@
       <c r="D222" s="1" t="s">
         <v>873</v>
       </c>
-      <c r="E222" s="1" t="s">
-        <v>872</v>
+      <c r="E222" s="2" t="s">
+        <v>2680</v>
       </c>
     </row>
     <row r="223" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -12162,8 +12451,8 @@
       <c r="D223" s="1" t="s">
         <v>877</v>
       </c>
-      <c r="E223" s="1" t="s">
-        <v>876</v>
+      <c r="E223" s="2" t="s">
+        <v>2681</v>
       </c>
     </row>
     <row r="224" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12179,8 +12468,8 @@
       <c r="D224" s="1" t="s">
         <v>881</v>
       </c>
-      <c r="E224" s="1" t="s">
-        <v>880</v>
+      <c r="E224" s="2" t="s">
+        <v>2682</v>
       </c>
     </row>
     <row r="225" spans="1:5" ht="102" x14ac:dyDescent="0.2">
@@ -12196,8 +12485,8 @@
       <c r="D225" s="1" t="s">
         <v>885</v>
       </c>
-      <c r="E225" s="1" t="s">
-        <v>884</v>
+      <c r="E225" s="2" t="s">
+        <v>2683</v>
       </c>
     </row>
     <row r="226" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12213,7 +12502,7 @@
       <c r="D226" s="1" t="s">
         <v>888</v>
       </c>
-      <c r="E226" s="1" t="s">
+      <c r="E226" s="2" t="s">
         <v>888</v>
       </c>
     </row>
@@ -12230,8 +12519,8 @@
       <c r="D227" s="1" t="s">
         <v>891</v>
       </c>
-      <c r="E227" s="1" t="s">
-        <v>891</v>
+      <c r="E227" s="2" t="s">
+        <v>2684</v>
       </c>
     </row>
     <row r="228" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12247,8 +12536,8 @@
       <c r="D228" s="1" t="s">
         <v>893</v>
       </c>
-      <c r="E228" s="1" t="s">
-        <v>893</v>
+      <c r="E228" s="2" t="s">
+        <v>2685</v>
       </c>
     </row>
     <row r="229" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12264,8 +12553,8 @@
       <c r="D229" s="1" t="s">
         <v>895</v>
       </c>
-      <c r="E229" s="1" t="s">
-        <v>895</v>
+      <c r="E229" s="2" t="s">
+        <v>2686</v>
       </c>
     </row>
     <row r="230" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12281,8 +12570,8 @@
       <c r="D230" s="1" t="s">
         <v>897</v>
       </c>
-      <c r="E230" s="1" t="s">
-        <v>897</v>
+      <c r="E230" s="2" t="s">
+        <v>2687</v>
       </c>
     </row>
     <row r="231" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12298,8 +12587,8 @@
       <c r="D231" s="1" t="s">
         <v>899</v>
       </c>
-      <c r="E231" s="1" t="s">
-        <v>899</v>
+      <c r="E231" s="2" t="s">
+        <v>2688</v>
       </c>
     </row>
     <row r="232" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12315,8 +12604,8 @@
       <c r="D232" s="1" t="s">
         <v>901</v>
       </c>
-      <c r="E232" s="1" t="s">
-        <v>901</v>
+      <c r="E232" s="2" t="s">
+        <v>2689</v>
       </c>
     </row>
     <row r="233" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12332,8 +12621,8 @@
       <c r="D233" s="1" t="s">
         <v>903</v>
       </c>
-      <c r="E233" s="1" t="s">
-        <v>903</v>
+      <c r="E233" s="2" t="s">
+        <v>2690</v>
       </c>
     </row>
     <row r="234" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -12791,8 +13080,8 @@
       <c r="D260" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="E260" s="1" t="s">
-        <v>539</v>
+      <c r="E260" s="2" t="s">
+        <v>2691</v>
       </c>
     </row>
     <row r="261" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -12808,8 +13097,8 @@
       <c r="D261" s="1" t="s">
         <v>992</v>
       </c>
-      <c r="E261" s="1" t="s">
-        <v>991</v>
+      <c r="E261" s="2" t="s">
+        <v>2692</v>
       </c>
     </row>
     <row r="262" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -12825,8 +13114,8 @@
       <c r="D262" s="1" t="s">
         <v>995</v>
       </c>
-      <c r="E262" s="1" t="s">
-        <v>995</v>
+      <c r="E262" s="2" t="s">
+        <v>2693</v>
       </c>
     </row>
     <row r="263" spans="1:5" ht="187" x14ac:dyDescent="0.2">
@@ -15698,8 +15987,8 @@
       <c r="D431" s="1" t="s">
         <v>1093</v>
       </c>
-      <c r="E431" s="1" t="s">
-        <v>1092</v>
+      <c r="E431" s="2" t="s">
+        <v>2499</v>
       </c>
     </row>
     <row r="432" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15715,8 +16004,8 @@
       <c r="D432" s="1" t="s">
         <v>1486</v>
       </c>
-      <c r="E432" s="1" t="s">
-        <v>1485</v>
+      <c r="E432" s="2" t="s">
+        <v>2694</v>
       </c>
     </row>
     <row r="433" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15732,8 +16021,8 @@
       <c r="D433" s="1" t="s">
         <v>1490</v>
       </c>
-      <c r="E433" s="1" t="s">
-        <v>1489</v>
+      <c r="E433" s="2" t="s">
+        <v>2695</v>
       </c>
     </row>
     <row r="434" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15749,8 +16038,8 @@
       <c r="D434" s="1" t="s">
         <v>1494</v>
       </c>
-      <c r="E434" s="1" t="s">
-        <v>1493</v>
+      <c r="E434" s="2" t="s">
+        <v>2696</v>
       </c>
     </row>
     <row r="435" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15766,8 +16055,8 @@
       <c r="D435" s="1" t="s">
         <v>1498</v>
       </c>
-      <c r="E435" s="1" t="s">
-        <v>1497</v>
+      <c r="E435" s="2" t="s">
+        <v>2697</v>
       </c>
     </row>
     <row r="436" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15783,8 +16072,8 @@
       <c r="D436" s="1" t="s">
         <v>1502</v>
       </c>
-      <c r="E436" s="1" t="s">
-        <v>1501</v>
+      <c r="E436" s="2" t="s">
+        <v>2698</v>
       </c>
     </row>
     <row r="437" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15800,8 +16089,8 @@
       <c r="D437" s="1" t="s">
         <v>1506</v>
       </c>
-      <c r="E437" s="1" t="s">
-        <v>1505</v>
+      <c r="E437" s="2" t="s">
+        <v>2699</v>
       </c>
     </row>
     <row r="438" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15817,8 +16106,8 @@
       <c r="D438" s="1" t="s">
         <v>1510</v>
       </c>
-      <c r="E438" s="1" t="s">
-        <v>1509</v>
+      <c r="E438" s="2" t="s">
+        <v>2700</v>
       </c>
     </row>
     <row r="439" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15834,8 +16123,8 @@
       <c r="D439" s="1" t="s">
         <v>1514</v>
       </c>
-      <c r="E439" s="1" t="s">
-        <v>1513</v>
+      <c r="E439" s="2" t="s">
+        <v>2701</v>
       </c>
     </row>
     <row r="440" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15851,8 +16140,8 @@
       <c r="D440" s="1" t="s">
         <v>1128</v>
       </c>
-      <c r="E440" s="1" t="s">
-        <v>163</v>
+      <c r="E440" s="2" t="s">
+        <v>2292</v>
       </c>
     </row>
     <row r="441" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15868,8 +16157,8 @@
       <c r="D441" s="1" t="s">
         <v>1132</v>
       </c>
-      <c r="E441" s="1" t="s">
-        <v>1131</v>
+      <c r="E441" s="2" t="s">
+        <v>2702</v>
       </c>
     </row>
     <row r="442" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15885,8 +16174,8 @@
       <c r="D442" s="1" t="s">
         <v>1522</v>
       </c>
-      <c r="E442" s="1" t="s">
-        <v>1521</v>
+      <c r="E442" s="2" t="s">
+        <v>2703</v>
       </c>
     </row>
     <row r="443" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -15902,8 +16191,8 @@
       <c r="D443" s="1" t="s">
         <v>1526</v>
       </c>
-      <c r="E443" s="1" t="s">
-        <v>1525</v>
+      <c r="E443" s="2" t="s">
+        <v>2704</v>
       </c>
     </row>
     <row r="444" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -15919,8 +16208,8 @@
       <c r="D444" s="1" t="s">
         <v>1530</v>
       </c>
-      <c r="E444" s="1" t="s">
-        <v>1529</v>
+      <c r="E444" s="2" t="s">
+        <v>2705</v>
       </c>
     </row>
     <row r="445" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15936,8 +16225,8 @@
       <c r="D445" s="1" t="s">
         <v>1148</v>
       </c>
-      <c r="E445" s="1" t="s">
-        <v>1147</v>
+      <c r="E445" s="2" t="s">
+        <v>2454</v>
       </c>
     </row>
     <row r="446" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15953,8 +16242,8 @@
       <c r="D446" s="1" t="s">
         <v>1152</v>
       </c>
-      <c r="E446" s="1" t="s">
-        <v>1151</v>
+      <c r="E446" s="2" t="s">
+        <v>2706</v>
       </c>
     </row>
     <row r="447" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -15970,7 +16259,7 @@
       <c r="D447" s="1" t="s">
         <v>1155</v>
       </c>
-      <c r="E447" s="1" t="s">
+      <c r="E447" s="2" t="s">
         <v>333</v>
       </c>
     </row>
@@ -15987,8 +16276,8 @@
       <c r="D448" s="1" t="s">
         <v>1159</v>
       </c>
-      <c r="E448" s="1" t="s">
-        <v>1158</v>
+      <c r="E448" s="2" t="s">
+        <v>2537</v>
       </c>
     </row>
     <row r="449" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -16004,7 +16293,7 @@
       <c r="D449" s="1" t="s">
         <v>1162</v>
       </c>
-      <c r="E449" s="1" t="s">
+      <c r="E449" s="2" t="s">
         <v>335</v>
       </c>
     </row>
@@ -16021,8 +16310,8 @@
       <c r="D450" s="1" t="s">
         <v>1166</v>
       </c>
-      <c r="E450" s="1" t="s">
-        <v>1165</v>
+      <c r="E450" s="2" t="s">
+        <v>2707</v>
       </c>
     </row>
     <row r="451" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -16038,7 +16327,7 @@
       <c r="D451" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="E451" s="1" t="s">
+      <c r="E451" s="2" t="s">
         <v>1169</v>
       </c>
     </row>
@@ -16055,8 +16344,8 @@
       <c r="D452" s="1" t="s">
         <v>1174</v>
       </c>
-      <c r="E452" s="1" t="s">
-        <v>2518</v>
+      <c r="E452" s="2" t="s">
+        <v>2708</v>
       </c>
     </row>
     <row r="453" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -16072,7 +16361,7 @@
       <c r="D453" s="1" t="s">
         <v>1178</v>
       </c>
-      <c r="E453" s="1" t="s">
+      <c r="E453" s="2" t="s">
         <v>1177</v>
       </c>
     </row>
@@ -16158,7 +16447,7 @@
         <v>1198</v>
       </c>
       <c r="E458" s="1" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="459" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16379,7 +16668,7 @@
         <v>1563</v>
       </c>
       <c r="E471" s="1" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="472" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -16396,7 +16685,7 @@
         <v>1567</v>
       </c>
       <c r="E472" s="1" t="s">
-        <v>2521</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="473" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16430,7 +16719,7 @@
         <v>1573</v>
       </c>
       <c r="E474" s="1" t="s">
-        <v>2522</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="475" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -16447,7 +16736,7 @@
         <v>1577</v>
       </c>
       <c r="E475" s="1" t="s">
-        <v>2523</v>
+        <v>2522</v>
       </c>
     </row>
     <row r="476" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -16464,7 +16753,7 @@
         <v>1581</v>
       </c>
       <c r="E476" s="1" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="477" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -16481,7 +16770,7 @@
         <v>1585</v>
       </c>
       <c r="E477" s="1" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="478" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16498,7 +16787,7 @@
         <v>1093</v>
       </c>
       <c r="E478" s="1" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="479" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -16515,7 +16804,7 @@
         <v>1591</v>
       </c>
       <c r="E479" s="1" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="480" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16532,7 +16821,7 @@
         <v>1490</v>
       </c>
       <c r="E480" s="1" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="481" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16549,7 +16838,7 @@
         <v>1597</v>
       </c>
       <c r="E481" s="1" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="482" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16566,7 +16855,7 @@
         <v>1601</v>
       </c>
       <c r="E482" s="1" t="s">
-        <v>2530</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="483" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16583,7 +16872,7 @@
         <v>1605</v>
       </c>
       <c r="E483" s="1" t="s">
-        <v>2531</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="484" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16600,7 +16889,7 @@
         <v>1609</v>
       </c>
       <c r="E484" s="1" t="s">
-        <v>2532</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="485" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16617,7 +16906,7 @@
         <v>1613</v>
       </c>
       <c r="E485" s="1" t="s">
-        <v>2533</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="486" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -16634,7 +16923,7 @@
         <v>1617</v>
       </c>
       <c r="E486" s="1" t="s">
-        <v>2534</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="487" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16685,7 +16974,7 @@
         <v>1625</v>
       </c>
       <c r="E489" s="1" t="s">
-        <v>2535</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="490" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -16702,7 +16991,7 @@
         <v>1629</v>
       </c>
       <c r="E490" s="1" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="491" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -16719,7 +17008,7 @@
         <v>1633</v>
       </c>
       <c r="E491" s="1" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="492" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -16787,7 +17076,7 @@
         <v>1159</v>
       </c>
       <c r="E495" s="1" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="496" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17178,7 +17467,7 @@
         <v>1666</v>
       </c>
       <c r="E518" s="1" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
     </row>
     <row r="519" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -17195,7 +17484,7 @@
         <v>1670</v>
       </c>
       <c r="E519" s="1" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="520" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17212,7 +17501,7 @@
         <v>1674</v>
       </c>
       <c r="E520" s="1" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="521" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -17229,7 +17518,7 @@
         <v>1678</v>
       </c>
       <c r="E521" s="1" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="522" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -17245,8 +17534,8 @@
       <c r="D522" s="1" t="s">
         <v>1682</v>
       </c>
-      <c r="E522" s="1" t="s">
-        <v>1681</v>
+      <c r="E522" s="2" t="s">
+        <v>2709</v>
       </c>
     </row>
     <row r="523" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -17262,8 +17551,8 @@
       <c r="D523" s="1" t="s">
         <v>1686</v>
       </c>
-      <c r="E523" s="1" t="s">
-        <v>1685</v>
+      <c r="E523" s="2" t="s">
+        <v>2710</v>
       </c>
     </row>
     <row r="524" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17279,8 +17568,8 @@
       <c r="D524" s="1" t="s">
         <v>1690</v>
       </c>
-      <c r="E524" s="1" t="s">
-        <v>1689</v>
+      <c r="E524" s="2" t="s">
+        <v>2711</v>
       </c>
     </row>
     <row r="525" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17296,8 +17585,8 @@
       <c r="D525" s="1" t="s">
         <v>1694</v>
       </c>
-      <c r="E525" s="1" t="s">
-        <v>1693</v>
+      <c r="E525" s="2" t="s">
+        <v>2712</v>
       </c>
     </row>
     <row r="526" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17313,8 +17602,8 @@
       <c r="D526" s="1" t="s">
         <v>1698</v>
       </c>
-      <c r="E526" s="1" t="s">
-        <v>1697</v>
+      <c r="E526" s="2" t="s">
+        <v>2713</v>
       </c>
     </row>
     <row r="527" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17330,8 +17619,8 @@
       <c r="D527" s="1" t="s">
         <v>1490</v>
       </c>
-      <c r="E527" s="1" t="s">
-        <v>1489</v>
+      <c r="E527" s="2" t="s">
+        <v>2695</v>
       </c>
     </row>
     <row r="528" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17347,8 +17636,8 @@
       <c r="D528" s="1" t="s">
         <v>1704</v>
       </c>
-      <c r="E528" s="1" t="s">
-        <v>1703</v>
+      <c r="E528" s="2" t="s">
+        <v>2714</v>
       </c>
     </row>
     <row r="529" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17364,8 +17653,8 @@
       <c r="D529" s="1" t="s">
         <v>1708</v>
       </c>
-      <c r="E529" s="1" t="s">
-        <v>1707</v>
+      <c r="E529" s="2" t="s">
+        <v>2715</v>
       </c>
     </row>
     <row r="530" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17381,8 +17670,8 @@
       <c r="D530" s="1" t="s">
         <v>1712</v>
       </c>
-      <c r="E530" s="1" t="s">
-        <v>1711</v>
+      <c r="E530" s="2" t="s">
+        <v>2716</v>
       </c>
     </row>
     <row r="531" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17398,8 +17687,8 @@
       <c r="D531" s="1" t="s">
         <v>1716</v>
       </c>
-      <c r="E531" s="1" t="s">
-        <v>1715</v>
+      <c r="E531" s="2" t="s">
+        <v>2717</v>
       </c>
     </row>
     <row r="532" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17415,8 +17704,8 @@
       <c r="D532" s="1" t="s">
         <v>1720</v>
       </c>
-      <c r="E532" s="1" t="s">
-        <v>1719</v>
+      <c r="E532" s="2" t="s">
+        <v>2718</v>
       </c>
     </row>
     <row r="533" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17432,8 +17721,8 @@
       <c r="D533" s="1" t="s">
         <v>1724</v>
       </c>
-      <c r="E533" s="1" t="s">
-        <v>1723</v>
+      <c r="E533" s="2" t="s">
+        <v>2719</v>
       </c>
     </row>
     <row r="534" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17449,8 +17738,8 @@
       <c r="D534" s="1" t="s">
         <v>1128</v>
       </c>
-      <c r="E534" s="1" t="s">
-        <v>163</v>
+      <c r="E534" s="2" t="s">
+        <v>2292</v>
       </c>
     </row>
     <row r="535" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17466,8 +17755,8 @@
       <c r="D535" s="1" t="s">
         <v>1132</v>
       </c>
-      <c r="E535" s="1" t="s">
-        <v>1131</v>
+      <c r="E535" s="2" t="s">
+        <v>2450</v>
       </c>
     </row>
     <row r="536" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17483,8 +17772,8 @@
       <c r="D536" s="1" t="s">
         <v>1732</v>
       </c>
-      <c r="E536" s="1" t="s">
-        <v>1731</v>
+      <c r="E536" s="2" t="s">
+        <v>2720</v>
       </c>
     </row>
     <row r="537" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17500,8 +17789,8 @@
       <c r="D537" s="1" t="s">
         <v>1736</v>
       </c>
-      <c r="E537" s="1" t="s">
-        <v>1735</v>
+      <c r="E537" s="2" t="s">
+        <v>2721</v>
       </c>
     </row>
     <row r="538" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -17518,7 +17807,7 @@
         <v>1740</v>
       </c>
       <c r="E538" s="1" t="s">
-        <v>1739</v>
+        <v>2722</v>
       </c>
     </row>
     <row r="539" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17773,7 +18062,7 @@
         <v>1202</v>
       </c>
       <c r="E553" s="1" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="554" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -17943,7 +18232,7 @@
         <v>1768</v>
       </c>
       <c r="E563" s="1" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="564" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -17960,7 +18249,7 @@
         <v>1772</v>
       </c>
       <c r="E564" s="1" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="565" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17977,7 +18266,7 @@
         <v>1776</v>
       </c>
       <c r="E565" s="1" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="566" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -17994,7 +18283,7 @@
         <v>1780</v>
       </c>
       <c r="E566" s="1" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="567" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -18011,7 +18300,7 @@
         <v>1784</v>
       </c>
       <c r="E567" s="1" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="568" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18028,7 +18317,7 @@
         <v>1788</v>
       </c>
       <c r="E568" s="1" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="569" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -18045,7 +18334,7 @@
         <v>1792</v>
       </c>
       <c r="E569" s="1" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="570" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18062,7 +18351,7 @@
         <v>1796</v>
       </c>
       <c r="E570" s="1" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="571" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -18079,7 +18368,7 @@
         <v>1800</v>
       </c>
       <c r="E571" s="1" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="572" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18096,7 +18385,7 @@
         <v>1804</v>
       </c>
       <c r="E572" s="1" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="573" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -18113,7 +18402,7 @@
         <v>1808</v>
       </c>
       <c r="E573" s="1" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="574" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18130,7 +18419,7 @@
         <v>1812</v>
       </c>
       <c r="E574" s="1" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="575" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -18147,7 +18436,7 @@
         <v>1816</v>
       </c>
       <c r="E575" s="1" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="576" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18164,7 +18453,7 @@
         <v>1820</v>
       </c>
       <c r="E576" s="1" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="577" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18181,7 +18470,7 @@
         <v>1824</v>
       </c>
       <c r="E577" s="1" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="578" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18198,7 +18487,7 @@
         <v>1828</v>
       </c>
       <c r="E578" s="1" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="579" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18215,7 +18504,7 @@
         <v>1832</v>
       </c>
       <c r="E579" s="1" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="580" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18232,7 +18521,7 @@
         <v>1836</v>
       </c>
       <c r="E580" s="1" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="581" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18249,7 +18538,7 @@
         <v>1840</v>
       </c>
       <c r="E581" s="1" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="582" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18283,7 +18572,7 @@
         <v>1846</v>
       </c>
       <c r="E583" s="1" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="584" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18402,7 +18691,7 @@
         <v>1856</v>
       </c>
       <c r="E590" s="1" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="591" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18453,7 +18742,7 @@
         <v>1864</v>
       </c>
       <c r="E593" s="1" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="594" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18470,7 +18759,7 @@
         <v>1868</v>
       </c>
       <c r="E594" s="1" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="595" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18487,7 +18776,7 @@
         <v>1872</v>
       </c>
       <c r="E595" s="1" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="596" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18504,7 +18793,7 @@
         <v>1876</v>
       </c>
       <c r="E596" s="1" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="597" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18538,7 +18827,7 @@
         <v>1882</v>
       </c>
       <c r="E598" s="1" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="599" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -18555,7 +18844,7 @@
         <v>1886</v>
       </c>
       <c r="E599" s="1" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
     </row>
     <row r="600" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18589,7 +18878,7 @@
         <v>1895</v>
       </c>
       <c r="E601" s="1" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="602" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18606,7 +18895,7 @@
         <v>1898</v>
       </c>
       <c r="E602" s="1" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="603" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18708,7 +18997,7 @@
         <v>1923</v>
       </c>
       <c r="E608" s="1" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="609" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18759,7 +19048,7 @@
         <v>1933</v>
       </c>
       <c r="E611" s="1" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="612" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18776,7 +19065,7 @@
         <v>1937</v>
       </c>
       <c r="E612" s="1" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="613" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18793,7 +19082,7 @@
         <v>1941</v>
       </c>
       <c r="E613" s="1" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="614" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -18946,7 +19235,7 @@
         <v>1856</v>
       </c>
       <c r="E622" s="1" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="623" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -18997,7 +19286,7 @@
         <v>1961</v>
       </c>
       <c r="E625" s="1" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="626" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19031,7 +19320,7 @@
         <v>1966</v>
       </c>
       <c r="E627" s="1" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="628" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19048,7 +19337,7 @@
         <v>1969</v>
       </c>
       <c r="E628" s="1" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="629" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19082,7 +19371,7 @@
         <v>1975</v>
       </c>
       <c r="E630" s="1" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="631" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19099,7 +19388,7 @@
         <v>1978</v>
       </c>
       <c r="E631" s="1" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="632" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19116,7 +19405,7 @@
         <v>1980</v>
       </c>
       <c r="E632" s="1" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="633" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19150,7 +19439,7 @@
         <v>1986</v>
       </c>
       <c r="E634" s="1" t="s">
-        <v>2583</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="635" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19184,7 +19473,7 @@
         <v>1994</v>
       </c>
       <c r="E636" s="1" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="637" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19201,7 +19490,7 @@
         <v>1998</v>
       </c>
       <c r="E637" s="1" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="638" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -19218,7 +19507,7 @@
         <v>2002</v>
       </c>
       <c r="E638" s="1" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="639" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19235,7 +19524,7 @@
         <v>2006</v>
       </c>
       <c r="E639" s="1" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="640" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19252,7 +19541,7 @@
         <v>2010</v>
       </c>
       <c r="E640" s="1" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="641" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19269,7 +19558,7 @@
         <v>2013</v>
       </c>
       <c r="E641" s="1" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="642" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19286,7 +19575,7 @@
         <v>2016</v>
       </c>
       <c r="E642" s="1" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="643" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19303,7 +19592,7 @@
         <v>2019</v>
       </c>
       <c r="E643" s="1" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="644" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -19320,7 +19609,7 @@
         <v>2022</v>
       </c>
       <c r="E644" s="1" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="645" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19337,7 +19626,7 @@
         <v>2026</v>
       </c>
       <c r="E645" s="1" t="s">
-        <v>2593</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="646" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19371,7 +19660,7 @@
         <v>2033</v>
       </c>
       <c r="E647" s="1" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
     </row>
     <row r="648" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19388,7 +19677,7 @@
         <v>2037</v>
       </c>
       <c r="E648" s="1" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
     </row>
     <row r="649" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19507,7 +19796,7 @@
         <v>2060</v>
       </c>
       <c r="E655" s="1" t="s">
-        <v>2596</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="656" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19524,7 +19813,7 @@
         <v>2064</v>
       </c>
       <c r="E656" s="1" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="657" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -19541,7 +19830,7 @@
         <v>2068</v>
       </c>
       <c r="E657" s="1" t="s">
-        <v>2598</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="658" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19575,7 +19864,7 @@
         <v>2074</v>
       </c>
       <c r="E659" s="1" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="660" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19592,7 +19881,7 @@
         <v>2078</v>
       </c>
       <c r="E660" s="1" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
     </row>
     <row r="661" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -19609,7 +19898,7 @@
         <v>2082</v>
       </c>
       <c r="E661" s="1" t="s">
-        <v>2601</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="662" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19643,7 +19932,7 @@
         <v>2088</v>
       </c>
       <c r="E663" s="1" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="664" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19711,7 +20000,7 @@
         <v>2102</v>
       </c>
       <c r="E667" s="1" t="s">
-        <v>2603</v>
+        <v>2602</v>
       </c>
     </row>
     <row r="668" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19745,7 +20034,7 @@
         <v>2111</v>
       </c>
       <c r="E669" s="1" t="s">
-        <v>2604</v>
+        <v>2603</v>
       </c>
     </row>
     <row r="670" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19779,7 +20068,7 @@
         <v>2120</v>
       </c>
       <c r="E671" s="1" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="672" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19813,7 +20102,7 @@
         <v>2128</v>
       </c>
       <c r="E673" s="1" t="s">
-        <v>2606</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="674" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -19830,7 +20119,7 @@
         <v>2131</v>
       </c>
       <c r="E674" s="1" t="s">
-        <v>2607</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="675" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19847,7 +20136,7 @@
         <v>2134</v>
       </c>
       <c r="E675" s="1" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="676" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19864,7 +20153,7 @@
         <v>1041</v>
       </c>
       <c r="E676" s="1" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="677" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19898,7 +20187,7 @@
         <v>2140</v>
       </c>
       <c r="E678" s="1" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="679" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19915,7 +20204,7 @@
         <v>2143</v>
       </c>
       <c r="E679" s="1" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="680" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -19932,7 +20221,7 @@
         <v>2146</v>
       </c>
       <c r="E680" s="1" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="681" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19949,7 +20238,7 @@
         <v>2149</v>
       </c>
       <c r="E681" s="1" t="s">
-        <v>2613</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="682" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -19983,7 +20272,7 @@
         <v>2154</v>
       </c>
       <c r="E683" s="1" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="684" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20017,7 +20306,7 @@
         <v>2160</v>
       </c>
       <c r="E685" s="1" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="686" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20034,7 +20323,7 @@
         <v>2163</v>
       </c>
       <c r="E686" s="1" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="687" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20051,7 +20340,7 @@
         <v>2165</v>
       </c>
       <c r="E687" s="1" t="s">
-        <v>2617</v>
+        <v>2616</v>
       </c>
     </row>
     <row r="688" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20068,7 +20357,7 @@
         <v>2168</v>
       </c>
       <c r="E688" s="1" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="689" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20085,7 +20374,7 @@
         <v>2170</v>
       </c>
       <c r="E689" s="1" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
     </row>
     <row r="690" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20102,7 +20391,7 @@
         <v>2173</v>
       </c>
       <c r="E690" s="1" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="691" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20119,7 +20408,7 @@
         <v>2176</v>
       </c>
       <c r="E691" s="1" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="692" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20136,7 +20425,7 @@
         <v>2179</v>
       </c>
       <c r="E692" s="1" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
     </row>
     <row r="693" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20153,7 +20442,7 @@
         <v>2182</v>
       </c>
       <c r="E693" s="1" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="694" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20187,7 +20476,7 @@
         <v>2186</v>
       </c>
       <c r="E695" s="1" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
     </row>
     <row r="696" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -20204,7 +20493,7 @@
         <v>2188</v>
       </c>
       <c r="E696" s="1" t="s">
-        <v>2625</v>
+        <v>2624</v>
       </c>
     </row>
     <row r="697" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20221,7 +20510,7 @@
         <v>2190</v>
       </c>
       <c r="E697" s="1" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="698" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20289,7 +20578,7 @@
         <v>2200</v>
       </c>
       <c r="E701" s="1" t="s">
-        <v>2627</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="702" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20340,7 +20629,7 @@
         <v>2206</v>
       </c>
       <c r="E704" s="1" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="705" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20357,7 +20646,7 @@
         <v>2208</v>
       </c>
       <c r="E705" s="1" t="s">
-        <v>2629</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="706" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20374,7 +20663,7 @@
         <v>2210</v>
       </c>
       <c r="E706" s="1" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
     </row>
     <row r="707" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20391,7 +20680,7 @@
         <v>2212</v>
       </c>
       <c r="E707" s="1" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="708" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20408,7 +20697,7 @@
         <v>2214</v>
       </c>
       <c r="E708" s="1" t="s">
-        <v>2632</v>
+        <v>2631</v>
       </c>
     </row>
     <row r="709" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -20425,7 +20714,7 @@
         <v>2217</v>
       </c>
       <c r="E709" s="1" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="710" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20459,7 +20748,7 @@
         <v>2221</v>
       </c>
       <c r="E711" s="1" t="s">
-        <v>2634</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="712" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20476,7 +20765,7 @@
         <v>2223</v>
       </c>
       <c r="E712" s="1" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="713" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20493,7 +20782,7 @@
         <v>2225</v>
       </c>
       <c r="E713" s="1" t="s">
-        <v>2636</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="714" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20561,7 +20850,7 @@
         <v>2235</v>
       </c>
       <c r="E717" s="1" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="718" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -20578,7 +20867,7 @@
         <v>2237</v>
       </c>
       <c r="E718" s="1" t="s">
-        <v>2638</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="719" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20595,7 +20884,7 @@
         <v>2239</v>
       </c>
       <c r="E719" s="1" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="720" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20612,7 +20901,7 @@
         <v>2242</v>
       </c>
       <c r="E720" s="1" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="721" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -20629,7 +20918,7 @@
         <v>2244</v>
       </c>
       <c r="E721" s="1" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="722" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20645,8 +20934,8 @@
       <c r="D722" s="1" t="s">
         <v>2246</v>
       </c>
-      <c r="E722" s="1" t="s">
-        <v>2246</v>
+      <c r="E722" s="2" t="s">
+        <v>2723</v>
       </c>
     </row>
     <row r="723" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20662,8 +20951,8 @@
       <c r="D723" s="1" t="s">
         <v>2249</v>
       </c>
-      <c r="E723" s="1" t="s">
-        <v>2248</v>
+      <c r="E723" s="2" t="s">
+        <v>2724</v>
       </c>
     </row>
     <row r="724" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20679,8 +20968,8 @@
       <c r="D724" s="1" t="s">
         <v>2251</v>
       </c>
-      <c r="E724" s="1" t="s">
-        <v>2251</v>
+      <c r="E724" s="2" t="s">
+        <v>2725</v>
       </c>
     </row>
     <row r="725" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20696,8 +20985,8 @@
       <c r="D725" s="1" t="s">
         <v>2253</v>
       </c>
-      <c r="E725" s="1" t="s">
-        <v>2253</v>
+      <c r="E725" s="2" t="s">
+        <v>2726</v>
       </c>
     </row>
     <row r="726" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20713,8 +21002,8 @@
       <c r="D726" s="1" t="s">
         <v>2255</v>
       </c>
-      <c r="E726" s="1" t="s">
-        <v>2255</v>
+      <c r="E726" s="2" t="s">
+        <v>2727</v>
       </c>
     </row>
     <row r="727" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20730,8 +21019,8 @@
       <c r="D727" s="1" t="s">
         <v>2257</v>
       </c>
-      <c r="E727" s="1" t="s">
-        <v>2257</v>
+      <c r="E727" s="2" t="s">
+        <v>2728</v>
       </c>
     </row>
     <row r="728" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -20747,8 +21036,8 @@
       <c r="D728" s="1" t="s">
         <v>2259</v>
       </c>
-      <c r="E728" s="1" t="s">
-        <v>2259</v>
+      <c r="E728" s="2" t="s">
+        <v>2729</v>
       </c>
     </row>
     <row r="729" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -20764,8 +21053,8 @@
       <c r="D729" s="1" t="s">
         <v>2261</v>
       </c>
-      <c r="E729" s="1" t="s">
-        <v>2261</v>
+      <c r="E729" s="2" t="s">
+        <v>2730</v>
       </c>
     </row>
     <row r="730" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20781,8 +21070,8 @@
       <c r="D730" s="1" t="s">
         <v>2263</v>
       </c>
-      <c r="E730" s="1" t="s">
-        <v>2263</v>
+      <c r="E730" s="2" t="s">
+        <v>2731</v>
       </c>
     </row>
     <row r="731" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20798,8 +21087,8 @@
       <c r="D731" s="1" t="s">
         <v>2266</v>
       </c>
-      <c r="E731" s="1" t="s">
-        <v>2265</v>
+      <c r="E731" s="2" t="s">
+        <v>2732</v>
       </c>
     </row>
     <row r="732" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -20815,8 +21104,8 @@
       <c r="D732" s="1" t="s">
         <v>2268</v>
       </c>
-      <c r="E732" s="1" t="s">
-        <v>2268</v>
+      <c r="E732" s="2" t="s">
+        <v>2733</v>
       </c>
     </row>
     <row r="733" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20832,8 +21121,8 @@
       <c r="D733" s="1" t="s">
         <v>2270</v>
       </c>
-      <c r="E733" s="1" t="s">
-        <v>2270</v>
+      <c r="E733" s="2" t="s">
+        <v>2734</v>
       </c>
     </row>
     <row r="734" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -20849,8 +21138,8 @@
       <c r="D734" s="1" t="s">
         <v>2273</v>
       </c>
-      <c r="E734" s="1" t="s">
-        <v>2272</v>
+      <c r="E734" s="2" t="s">
+        <v>2735</v>
       </c>
     </row>
   </sheetData>

</xml_diff>